<commit_message>
Add Nozzleworks logo to quote spreadsheet header
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CYtC1oymXdLojNWgt7AC92
</commit_message>
<xml_diff>
--- a/quote-template/Quote_Template.xlsx
+++ b/quote-template/Quote_Template.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="165" formatCode="#,##0.00;(#,##0.00);&quot;&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;NZD&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,12 +51,6 @@
       <name val="Calibri"/>
       <color rgb="007F7F7F"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00404040"/>
-      <sz val="16"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -134,23 +128,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -169,25 +160,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,7 +194,7 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -297,11 +288,6 @@
     <author>Template</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0">
-      <text>
-        <t>Logo placeholder - replace with the Nozzleworks logo (Insert &gt; Pictures).</t>
-      </text>
-    </comment>
     <comment ref="I2" authorId="0" shapeId="0">
       <text>
         <t>NZ GST 15% (Inland Revenue).</t>
@@ -309,6 +295,36 @@
     </comment>
   </commentList>
 </comments>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2000250" cy="257175"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -615,222 +631,217 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>NOZZLEWORKS</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Quotation</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Settings</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>GST 144-375-106</t>
         </is>
       </c>
-      <c r="D2" s="5">
+      <c r="D2" s="4">
         <f>"# "&amp;F3</f>
         <v/>
       </c>
-      <c r="H2" s="6" t="inlineStr">
+      <c r="H2" s="5" t="inlineStr">
         <is>
           <t>GST rate</t>
         </is>
       </c>
-      <c r="I2" s="7" t="n">
+      <c r="I2" s="6" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t>info@nozzleworks.co.nz</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Quote No :</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>QT-26001</t>
         </is>
       </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Validity (days)</t>
         </is>
       </c>
-      <c r="I3" s="9" t="n">
+      <c r="I3" s="8" t="n">
         <v>30</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>nozzleworks.co.nz</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>Quote Date :</t>
         </is>
       </c>
-      <c r="F4" s="10">
+      <c r="F4" s="9">
         <f>TODAY()</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Expiry Date :</t>
         </is>
       </c>
-      <c r="F5" s="10">
+      <c r="F5" s="9">
         <f>F4+$I$3</f>
         <v/>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Edit: quote no., quote date, customer,</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="H6" s="11" t="inlineStr">
+      <c r="H6" s="10" t="inlineStr">
         <is>
           <t>subject, part no., description, qty,</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Client Full Name</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr">
+      <c r="H7" s="10" t="inlineStr">
         <is>
           <t>UoM, unit price, notes and terms.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Job Title</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>#, sub-totals, GST, total and expiry</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Company Name</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>date are formulas - don't type over.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>Hide unused item rows before printing.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Subject :</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>Subject line</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Part No. &amp; Description</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>UoM</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Unit Price</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Sub-Total</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15">
+      <c r="A14" s="14">
         <f>IF(OR(B14&lt;&gt;"",C14&lt;&gt;""),1,"")</f>
         <v/>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>NW-EXAMPLE-01</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="6" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>pcs</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="17" t="n">
         <v>125</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="17">
         <f>IF(OR(C14="",E14=""),"",C14*E14)</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Example description - replace or delete this item</t>
         </is>
@@ -838,269 +849,269 @@
     </row>
     <row r="16" ht="6" customHeight="1"/>
     <row r="17">
-      <c r="A17" s="15">
+      <c r="A17" s="14">
         <f>IF(OR(B17&lt;&gt;"",C17&lt;&gt;""),2,"")</f>
         <v/>
       </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="17" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="18" t="n"/>
-      <c r="F17" s="18">
+      <c r="B17" s="15" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17">
         <f>IF(OR(C17="",E17=""),"",C17*E17)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="19" t="n"/>
+      <c r="B18" s="18" t="n"/>
     </row>
     <row r="19" ht="6" customHeight="1"/>
     <row r="20">
-      <c r="A20" s="15">
+      <c r="A20" s="14">
         <f>IF(OR(B20&lt;&gt;"",C20&lt;&gt;""),3,"")</f>
         <v/>
       </c>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="17" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="18" t="n"/>
-      <c r="F20" s="18">
+      <c r="B20" s="15" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17">
         <f>IF(OR(C20="",E20=""),"",C20*E20)</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="19" t="n"/>
+      <c r="B21" s="18" t="n"/>
     </row>
     <row r="22" ht="6" customHeight="1"/>
     <row r="23">
-      <c r="A23" s="15">
+      <c r="A23" s="14">
         <f>IF(OR(B23&lt;&gt;"",C23&lt;&gt;""),4,"")</f>
         <v/>
       </c>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="18" t="n"/>
-      <c r="F23" s="18">
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="16" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17">
         <f>IF(OR(C23="",E23=""),"",C23*E23)</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="19" t="n"/>
+      <c r="B24" s="18" t="n"/>
     </row>
     <row r="25" ht="6" customHeight="1"/>
     <row r="26">
-      <c r="A26" s="15">
+      <c r="A26" s="14">
         <f>IF(OR(B26&lt;&gt;"",C26&lt;&gt;""),5,"")</f>
         <v/>
       </c>
-      <c r="B26" s="16" t="n"/>
-      <c r="C26" s="17" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="18" t="n"/>
-      <c r="F26" s="18">
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17">
         <f>IF(OR(C26="",E26=""),"",C26*E26)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="19" t="n"/>
+      <c r="B27" s="18" t="n"/>
     </row>
     <row r="28" ht="6" customHeight="1"/>
     <row r="29">
-      <c r="A29" s="15">
+      <c r="A29" s="14">
         <f>IF(OR(B29&lt;&gt;"",C29&lt;&gt;""),6,"")</f>
         <v/>
       </c>
-      <c r="B29" s="16" t="n"/>
-      <c r="C29" s="17" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="18" t="n"/>
-      <c r="F29" s="18">
+      <c r="B29" s="15" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17">
         <f>IF(OR(C29="",E29=""),"",C29*E29)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="19" t="n"/>
+      <c r="B30" s="18" t="n"/>
     </row>
     <row r="31" ht="6" customHeight="1"/>
     <row r="32">
-      <c r="A32" s="15">
+      <c r="A32" s="14">
         <f>IF(OR(B32&lt;&gt;"",C32&lt;&gt;""),7,"")</f>
         <v/>
       </c>
-      <c r="B32" s="16" t="n"/>
-      <c r="C32" s="17" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="18" t="n"/>
-      <c r="F32" s="18">
+      <c r="B32" s="15" t="n"/>
+      <c r="C32" s="16" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17">
         <f>IF(OR(C32="",E32=""),"",C32*E32)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="19" t="n"/>
+      <c r="B33" s="18" t="n"/>
     </row>
     <row r="34" ht="6" customHeight="1"/>
     <row r="35">
-      <c r="A35" s="15">
+      <c r="A35" s="14">
         <f>IF(OR(B35&lt;&gt;"",C35&lt;&gt;""),8,"")</f>
         <v/>
       </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="17" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="18" t="n"/>
-      <c r="F35" s="18">
+      <c r="B35" s="15" t="n"/>
+      <c r="C35" s="16" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17">
         <f>IF(OR(C35="",E35=""),"",C35*E35)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="19" t="n"/>
+      <c r="B36" s="18" t="n"/>
     </row>
     <row r="37" ht="6" customHeight="1"/>
     <row r="38">
-      <c r="A38" s="15">
+      <c r="A38" s="14">
         <f>IF(OR(B38&lt;&gt;"",C38&lt;&gt;""),9,"")</f>
         <v/>
       </c>
-      <c r="B38" s="16" t="n"/>
-      <c r="C38" s="17" t="n"/>
-      <c r="D38" s="6" t="n"/>
-      <c r="E38" s="18" t="n"/>
-      <c r="F38" s="18">
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="16" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17">
         <f>IF(OR(C38="",E38=""),"",C38*E38)</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="19" t="n"/>
+      <c r="B39" s="18" t="n"/>
     </row>
     <row r="40" ht="6" customHeight="1"/>
     <row r="41">
-      <c r="A41" s="15">
+      <c r="A41" s="14">
         <f>IF(OR(B41&lt;&gt;"",C41&lt;&gt;""),10,"")</f>
         <v/>
       </c>
-      <c r="B41" s="16" t="n"/>
-      <c r="C41" s="17" t="n"/>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="18" t="n"/>
-      <c r="F41" s="18">
+      <c r="B41" s="15" t="n"/>
+      <c r="C41" s="16" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="17" t="n"/>
+      <c r="F41" s="17">
         <f>IF(OR(C41="",E41=""),"",C41*E41)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="19" t="n"/>
+      <c r="B42" s="18" t="n"/>
     </row>
     <row r="44" ht="6" customHeight="1">
-      <c r="A44" s="20" t="n"/>
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="20" t="n"/>
-      <c r="D44" s="20" t="n"/>
-      <c r="E44" s="20" t="n"/>
-      <c r="F44" s="20" t="n"/>
+      <c r="A44" s="19" t="n"/>
+      <c r="B44" s="19" t="n"/>
+      <c r="C44" s="19" t="n"/>
+      <c r="D44" s="19" t="n"/>
+      <c r="E44" s="19" t="n"/>
+      <c r="F44" s="19" t="n"/>
     </row>
     <row r="45">
-      <c r="E45" s="8" t="inlineStr">
+      <c r="E45" s="7" t="inlineStr">
         <is>
           <t>Sub Total</t>
         </is>
       </c>
-      <c r="F45" s="21">
+      <c r="F45" s="20">
         <f>SUM(F14:F42)</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="E46" s="8">
+      <c r="E46" s="7">
         <f>"GST ("&amp;TEXT($I$2,"0%")&amp;")"</f>
         <v/>
       </c>
-      <c r="F46" s="21">
+      <c r="F46" s="20">
         <f>ROUND(F45*$I$2,2)</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="6" customHeight="1">
-      <c r="D47" s="20" t="n"/>
-      <c r="E47" s="20" t="n"/>
-      <c r="F47" s="20" t="n"/>
+      <c r="D47" s="19" t="n"/>
+      <c r="E47" s="19" t="n"/>
+      <c r="F47" s="19" t="n"/>
     </row>
     <row r="48">
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E48" s="21" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="F48" s="23">
+      <c r="F48" s="22">
         <f>F45+F46</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="24" t="inlineStr">
+      <c r="A50" s="23" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>Delivery: approx. 3 weeks</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="inlineStr">
+      <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Shipping terms: ex-works.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Prices are GST exclusive.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="inlineStr">
+      <c r="A54" s="5" t="inlineStr">
         <is>
           <t>Order by emailing to Info@NozzleWorks.co.nz.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="24" t="inlineStr">
+      <c r="A56" s="23" t="inlineStr">
         <is>
           <t>Terms &amp; Conditions</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>Shipping: Ex works</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="inlineStr">
+      <c r="A58" s="5" t="inlineStr">
         <is>
           <t>Payment: On account, 20th month following date of invoice</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="6">
+      <c r="A59" s="5">
         <f>"Validity: "&amp;$I$3&amp;" days"</f>
         <v/>
       </c>
@@ -1188,6 +1199,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>